<commit_message>
Add the candidate records Q3 and I3 of the empirical study
Translate the titles written in Chinese in all screening tables.
</commit_message>
<xml_diff>
--- a/empirical-study/manual-screening.xlsx
+++ b/empirical-study/manual-screening.xlsx
@@ -7614,7 +7614,7 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>[BUG] Claw Run现在无法部署。是否版本太低。</t>
+          <t>[BUG] Claw Run can no longer be deployed. Is the version too old? [translated]</t>
         </is>
       </c>
       <c r="E225" t="inlineStr">
@@ -12254,7 +12254,7 @@
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>pod多容器申请vGPU调度失败</t>
+          <t>Scheduling fails when multiple containers of a Pod request vGPUs [translated]</t>
         </is>
       </c>
       <c r="E370" t="inlineStr">
@@ -13150,7 +13150,7 @@
       </c>
       <c r="D398" t="inlineStr">
         <is>
-          <t>claw.cloud用安装gpt-load报错</t>
+          <t>Error when installing gpt-load on claw.cloud [translated]</t>
         </is>
       </c>
       <c r="E398" t="inlineStr">
@@ -13598,7 +13598,7 @@
       </c>
       <c r="D412" t="inlineStr">
         <is>
-          <t>ClawCloud 1.0.9 部署不成功。</t>
+          <t>Deployment on ClawCloud 1.0.9 fails. [translated]</t>
         </is>
       </c>
       <c r="E412" t="inlineStr">

</xml_diff>